<commit_message>
fix: align etl pipeline and reports parser with new consolidated column layout of sheet QC10002-R02
</commit_message>
<xml_diff>
--- a/public/DataExtract/2025品檢報表統計.xlsx
+++ b/public/DataExtract/2025品檢報表統計.xlsx
@@ -3472,42 +3472,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:N15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>原物料進料品檢</v>
       </c>
-      <c r="B1" t="str">
-        <v/>
-      </c>
-      <c r="C1" t="str">
-        <v/>
-      </c>
-      <c r="D1" t="str">
-        <v/>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v/>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v/>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v>物料</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3517,54 +3487,39 @@
         <v>原料</v>
       </c>
       <c r="C2" t="str">
-        <v>物料</v>
+        <v>B膠</v>
       </c>
       <c r="D2" t="str">
+        <v>收縮膜</v>
+      </c>
+      <c r="E2" t="str">
+        <v>色粉</v>
+      </c>
+      <c r="F2" t="str">
+        <v>空白包裝袋</v>
+      </c>
+      <c r="G2" t="str">
+        <v>空白感壓紙</v>
+      </c>
+      <c r="H2" t="str">
+        <v>塑膠袋</v>
+      </c>
+      <c r="I2" t="str">
+        <v>塑膠袋40*50</v>
+      </c>
+      <c r="J2" t="str">
         <v>紙箱</v>
       </c>
-      <c r="E2" t="str">
+      <c r="K2" t="str">
         <v>過濾網連蓋</v>
       </c>
-      <c r="F2" t="str">
+      <c r="L2" t="str">
         <v>標籤</v>
       </c>
-      <c r="G2" t="str">
+      <c r="M2" t="str">
         <v>射出D</v>
       </c>
-      <c r="H2" t="str">
-        <v>小計</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v>月份</v>
-      </c>
-      <c r="L2" t="str">
-        <v>B膠</v>
-      </c>
-      <c r="M2" t="str">
-        <v>收縮膜</v>
-      </c>
       <c r="N2" t="str">
-        <v>色粉</v>
-      </c>
-      <c r="O2" t="str">
-        <v>空白包裝袋</v>
-      </c>
-      <c r="P2" t="str">
-        <v>空白感壓紙</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>塑膠袋</v>
-      </c>
-      <c r="R2" t="str">
-        <v>塑膠袋40*50</v>
-      </c>
-      <c r="S2" t="str">
         <v>小計</v>
       </c>
     </row>
@@ -3576,55 +3531,40 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
         <v>18</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
         <v>209</v>
       </c>
-      <c r="H3">
+      <c r="N3">
         <v>257</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-      <c r="N3">
-        <v>1</v>
-      </c>
-      <c r="O3">
-        <v>1</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>3</v>
-      </c>
-      <c r="R3">
-        <v>3</v>
-      </c>
-      <c r="S3">
-        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -3635,55 +3575,40 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
         <v>5</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4">
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
         <v>185</v>
       </c>
-      <c r="H4">
+      <c r="N4">
         <v>212</v>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>3</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>1</v>
-      </c>
-      <c r="Q4">
-        <v>1</v>
-      </c>
-      <c r="R4">
-        <v>2</v>
-      </c>
-      <c r="S4">
-        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -3694,55 +3619,40 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
         <v>5</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
         <v>5</v>
       </c>
-      <c r="G5">
+      <c r="M5">
         <v>233</v>
       </c>
-      <c r="H5">
+      <c r="N5">
         <v>271</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>3</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>1</v>
-      </c>
-      <c r="S5">
-        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -3753,55 +3663,40 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
         <v>3</v>
       </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
         <v>228</v>
       </c>
-      <c r="H6">
+      <c r="N6">
         <v>258</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3812,55 +3707,40 @@
         <v>15</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
         <v>4</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
         <v>219</v>
       </c>
-      <c r="H7">
+      <c r="N7">
         <v>245</v>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7">
-        <v>5</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
-      <c r="O7">
-        <v>2</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>3</v>
-      </c>
-      <c r="R7">
-        <v>1</v>
-      </c>
-      <c r="S7">
-        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -3871,55 +3751,40 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
         <v>6</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>2</v>
-      </c>
-      <c r="G8">
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8">
         <v>251</v>
       </c>
-      <c r="H8">
+      <c r="N8">
         <v>269</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
-      <c r="K8">
-        <v>6</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>1</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
-        <v>0</v>
-      </c>
-      <c r="R8">
-        <v>1</v>
-      </c>
-      <c r="S8">
-        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -3930,55 +3795,40 @@
         <v>24</v>
       </c>
       <c r="C9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>3</v>
+      </c>
+      <c r="J9">
         <v>5</v>
       </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
         <v>3</v>
       </c>
-      <c r="G9">
+      <c r="M9">
         <v>218</v>
       </c>
-      <c r="H9">
+      <c r="N9">
         <v>256</v>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
-      <c r="K9">
-        <v>7</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
-        <v>3</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>0</v>
-      </c>
-      <c r="Q9">
-        <v>0</v>
-      </c>
-      <c r="R9">
-        <v>3</v>
-      </c>
-      <c r="S9">
-        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -3992,52 +3842,37 @@
         <v>12</v>
       </c>
       <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
         <v>6</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>2</v>
-      </c>
-      <c r="G10">
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10">
         <v>193</v>
       </c>
-      <c r="H10">
+      <c r="N10">
         <v>233</v>
-      </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10">
-        <v>8</v>
-      </c>
-      <c r="L10">
-        <v>12</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -4048,55 +3883,40 @@
         <v>31</v>
       </c>
       <c r="C11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>2</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
         <v>5</v>
       </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
         <v>3</v>
       </c>
-      <c r="G11">
+      <c r="M11">
         <v>183</v>
       </c>
-      <c r="H11">
+      <c r="N11">
         <v>226</v>
-      </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v/>
-      </c>
-      <c r="K11">
-        <v>9</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <v>2</v>
-      </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
-        <v>0</v>
-      </c>
-      <c r="Q11">
-        <v>2</v>
-      </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -4107,55 +3927,40 @@
         <v>20</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
         <v>8</v>
       </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
         <v>211</v>
       </c>
-      <c r="H12">
+      <c r="N12">
         <v>241</v>
-      </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
-      <c r="J12" t="str">
-        <v/>
-      </c>
-      <c r="K12">
-        <v>10</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>2</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
-        <v>0</v>
-      </c>
-      <c r="Q12">
-        <v>0</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -4166,55 +3971,40 @@
         <v>30</v>
       </c>
       <c r="C13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
         <v>5</v>
       </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
         <v>198</v>
       </c>
-      <c r="H13">
+      <c r="N13">
         <v>245</v>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
-      <c r="K13">
-        <v>11</v>
-      </c>
-      <c r="L13">
-        <v>11</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>1</v>
-      </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>0</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -4228,52 +4018,37 @@
         <v>0</v>
       </c>
       <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
         <v>7</v>
       </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
         <v>4</v>
       </c>
-      <c r="G14">
+      <c r="M14">
         <v>168</v>
       </c>
-      <c r="H14">
+      <c r="N14">
         <v>193</v>
-      </c>
-      <c r="I14" t="str">
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
-      <c r="K14">
-        <v>12</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>0</v>
-      </c>
-      <c r="Q14">
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -4284,60 +4059,45 @@
         <v>242</v>
       </c>
       <c r="C15">
-        <v>67</v>
+        <v>23</v>
       </c>
       <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>17</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>9</v>
+      </c>
+      <c r="I15">
+        <v>11</v>
+      </c>
+      <c r="J15">
         <v>61</v>
       </c>
-      <c r="E15">
+      <c r="K15">
         <v>18</v>
       </c>
-      <c r="F15">
+      <c r="L15">
         <v>22</v>
       </c>
-      <c r="G15">
+      <c r="M15">
         <v>2496</v>
       </c>
-      <c r="H15">
+      <c r="N15">
         <v>2906</v>
-      </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
-      <c r="K15" t="str">
-        <v>小計</v>
-      </c>
-      <c r="L15">
-        <v>23</v>
-      </c>
-      <c r="M15">
-        <v>3</v>
-      </c>
-      <c r="N15">
-        <v>17</v>
-      </c>
-      <c r="O15">
-        <v>3</v>
-      </c>
-      <c r="P15">
-        <v>1</v>
-      </c>
-      <c r="Q15">
-        <v>9</v>
-      </c>
-      <c r="R15">
-        <v>11</v>
-      </c>
-      <c r="S15">
-        <v>67</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>